<commit_message>
Apply the verification findings: NCDOT rounding chart, TEAAS rounding, workbook notes
AADT workbook: per-leg estimates now round per the NCDOT/AASHTO AADT
rounding chart; the entering AADT is rounded to the nearest hundred as
TEAAS Chapter 8 directs (12,050 -> 12,100 vpd, 44.17 MEV) and drives the
exposure and crash rate; the middle-year comment follows each sheet's
dates, the crash-count label no longer repeats the input, and every
formula reading the Stations sheet is green. README, aadt.json,
aadt_calculation.txt, the AADT map box and the CalculatedAADT note use
the same wording; README reconciles the TEAAS-entered 5-yr ADT 15,200.
Collision diagram sheet: the M&D Quick Stop label sits clear of the
frontage arc (drawn at 0.9); check_relabel.py matches with a tolerance.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012AMZ23B9M2AjrQa7UP3LHH
</commit_message>
<xml_diff>
--- a/HSIP/41000079736/41000079736_AADT.xlsx
+++ b/HSIP/41000079736/41000079736_AADT.xlsx
@@ -35,7 +35,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Year containing the midpoint date of the study period (9/1/2016-8/31/2026 -&gt; 1 Sep 2021 -&gt; 2021).</t>
+          <t xml:space="preserve">Year containing the midpoint date of the study period 09/01/2016-08/31/2026: =YEAR(B4+(B5-B4)/2).</t>
         </r>
       </text>
     </comment>
@@ -47,7 +47,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Crash count from the TEAAS Intersection Analysis Report, 10-yr report, 29 crashes; used only for the crash rate.</t>
+          <t xml:space="preserve">Crash count from the TEAAS 10-yr Intersection Analysis Report for this study period; used only for the crash rate.</t>
         </r>
       </text>
     </comment>
@@ -69,7 +69,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Year containing the midpoint date of the study period (9/1/2016-8/31/2026 -&gt; 1 Sep 2021 -&gt; 2021).</t>
+          <t xml:space="preserve">Year containing the midpoint date of the study period 09/01/2021-08/31/2026: =YEAR(B4+(B5-B4)/2).</t>
         </r>
       </text>
     </comment>
@@ -81,7 +81,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Crash count from the TEAAS Intersection Analysis Report, 5-yr report, 22 crashes; used only for the crash rate.</t>
+          <t xml:space="preserve">Crash count from the TEAAS 5-yr Intersection Analysis Report for this study period; used only for the crash rate.</t>
         </r>
       </text>
     </comment>
@@ -90,12 +90,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="56">
   <si>
     <t xml:space="preserve">Entering AADT for the 10-yr study - Order# 41000079736, NC 180/NC 226 (S Post Rd) at SR 1103, Cleveland County</t>
   </si>
   <si>
-    <t xml:space="preserve">Method: each leg uses its NCDOT station count for the middle year of the study period. A leg with no count for that year gets a straight-line estimate between the nearest earlier and later published counts, rounded the way NCDOT publishes AADT (nearest 100 at 1,000 vpd and over, nearest 10 below) and marked "estimate". Entering AADT = sum of the four leg AADTs / 2. Exposure (MEV) = entering AADT x 365 x years / 1,000,000. Blue cells are inputs; everything else is a formula reading the Stations sheet.</t>
+    <t xml:space="preserve">Method: each leg uses its NCDOT station count for the middle year of the study period. A leg with no count for that year gets a straight-line estimate between the nearest earlier and later published counts, rounded per the NCDOT/AASHTO AADT rounding chart (nearest 10 below 100, 50 for 100-999, 100 for 1,000-9,999, 500 for 10,000-99,999, 1,000 above) and marked "estimate". Entering AADT = sum of the four leg AADTs / 2, rounded to the nearest hundred as TEAAS Chapter 8 directs. Exposure (MEV) = rounded entering AADT x 365 x years / 1,000,000. Blue cells are inputs; everything else is a formula reading the Stations sheet.</t>
   </si>
   <si>
     <t xml:space="preserve">Study period start</t>
@@ -110,7 +110,7 @@
     <t xml:space="preserve">Study length (years)</t>
   </si>
   <si>
-    <t xml:space="preserve">Crashes in the study period (10-yr report, 29 crashes)</t>
+    <t xml:space="preserve">Crashes in the study period (TEAAS 10-yr Intersection Analysis Report)</t>
   </si>
   <si>
     <t xml:space="preserve">Leg</t>
@@ -149,7 +149,7 @@
     <t xml:space="preserve">Straight-line estimate for the middle year, unrounded</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimate rounded as NCDOT publishes</t>
+    <t xml:space="preserve">Estimate rounded per the NCDOT/AASHTO AADT rounding chart</t>
   </si>
   <si>
     <t xml:space="preserve">AADT used for the middle year (vpd)</t>
@@ -167,7 +167,10 @@
     <t xml:space="preserve">Entering AADT = sum / 2 (vpd)</t>
   </si>
   <si>
-    <t xml:space="preserve">Exposure, million entering vehicles = AADT x 365 x years / 1,000,000</t>
+    <t xml:space="preserve">Entering AADT rounded to the nearest hundred (TEAAS Chapter 8) (vpd)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exposure, million entering vehicles = rounded AADT x 365 x years / 1,000,000</t>
   </si>
   <si>
     <t xml:space="preserve">Crash rate (crashes per million entering vehicles)</t>
@@ -251,7 +254,7 @@
     <t xml:space="preserve">Entering AADT for the 5-yr study - Order# 41000079736, NC 180/NC 226 (S Post Rd) at SR 1103, Cleveland County</t>
   </si>
   <si>
-    <t xml:space="preserve">Crashes in the study period (5-yr report, 22 crashes)</t>
+    <t xml:space="preserve">Crashes in the study period (TEAAS 5-yr Intersection Analysis Report)</t>
   </si>
   <si>
     <t xml:space="preserve">Used on the collision diagram and in the study: no (check only)</t>
@@ -425,7 +428,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -470,15 +473,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="169" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -778,7 +785,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
@@ -1009,40 +1016,40 @@
       <c r="A18" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="11" t="n">
-        <f aca="false">IFERROR(IF(B17&gt;=1000,ROUND(B17,-2),ROUND(B17,-1)),"")</f>
+      <c r="B18" s="14" t="n">
+        <f aca="false">IFERROR(IF(B17&gt;99999,ROUND(B17,-3),IF(B17&gt;=10000,ROUND(B17/500,0)*500,IF(B17&gt;=1000,ROUND(B17,-2),IF(B17&gt;=100,ROUND(B17/50,0)*50,ROUND(B17,-1))))),"")</f>
         <v>11500</v>
       </c>
-      <c r="C18" s="11" t="n">
-        <f aca="false">IFERROR(IF(C17&gt;=1000,ROUND(C17,-2),ROUND(C17,-1)),"")</f>
-        <v>10200</v>
-      </c>
-      <c r="D18" s="11" t="n">
-        <f aca="false">IFERROR(IF(D17&gt;=1000,ROUND(D17,-2),ROUND(D17,-1)),"")</f>
+      <c r="C18" s="14" t="n">
+        <f aca="false">IFERROR(IF(C17&gt;99999,ROUND(C17,-3),IF(C17&gt;=10000,ROUND(C17/500,0)*500,IF(C17&gt;=1000,ROUND(C17,-2),IF(C17&gt;=100,ROUND(C17/50,0)*50,ROUND(C17,-1))))),"")</f>
+        <v>10000</v>
+      </c>
+      <c r="D18" s="14" t="n">
+        <f aca="false">IFERROR(IF(D17&gt;99999,ROUND(D17,-3),IF(D17&gt;=10000,ROUND(D17/500,0)*500,IF(D17&gt;=1000,ROUND(D17,-2),IF(D17&gt;=100,ROUND(D17/50,0)*50,ROUND(D17,-1))))),"")</f>
         <v>1400</v>
       </c>
-      <c r="E18" s="11" t="n">
-        <f aca="false">IFERROR(IF(E17&gt;=1000,ROUND(E17,-2),ROUND(E17,-1)),"")</f>
+      <c r="E18" s="14" t="n">
+        <f aca="false">IFERROR(IF(E17&gt;99999,ROUND(E17,-3),IF(E17&gt;=10000,ROUND(E17/500,0)*500,IF(E17&gt;=1000,ROUND(E17,-2),IF(E17&gt;=100,ROUND(E17/50,0)*50,ROUND(E17,-1))))),"")</f>
         <v>1100</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="11" t="n">
+      <c r="B19" s="14" t="n">
         <f aca="false">IF(B12&lt;&gt;"",B12,B18)</f>
         <v>11000</v>
       </c>
-      <c r="C19" s="11" t="n">
+      <c r="C19" s="14" t="n">
         <f aca="false">IF(C12&lt;&gt;"",C12,C18)</f>
         <v>10500</v>
       </c>
-      <c r="D19" s="11" t="n">
+      <c r="D19" s="14" t="n">
         <f aca="false">IF(D12&lt;&gt;"",D12,D18)</f>
         <v>1400</v>
       </c>
-      <c r="E19" s="11" t="n">
+      <c r="E19" s="14" t="n">
         <f aca="false">IF(E12&lt;&gt;"",E12,E18)</f>
         <v>1200</v>
       </c>
@@ -1051,19 +1058,19 @@
       <c r="A20" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="15" t="str">
+      <c r="B20" s="16" t="str">
         <f aca="false">IF(B12&lt;&gt;"","count",IF(B18&lt;&gt;"","estimate","no data"))</f>
         <v>count</v>
       </c>
-      <c r="C20" s="15" t="str">
+      <c r="C20" s="16" t="str">
         <f aca="false">IF(C12&lt;&gt;"","count",IF(C18&lt;&gt;"","estimate","no data"))</f>
         <v>count</v>
       </c>
-      <c r="D20" s="15" t="str">
+      <c r="D20" s="16" t="str">
         <f aca="false">IF(D12&lt;&gt;"","count",IF(D18&lt;&gt;"","estimate","no data"))</f>
         <v>estimate</v>
       </c>
-      <c r="E20" s="15" t="str">
+      <c r="E20" s="16" t="str">
         <f aca="false">IF(E12&lt;&gt;"","count",IF(E18&lt;&gt;"","estimate","no data"))</f>
         <v>count</v>
       </c>
@@ -1072,19 +1079,19 @@
       <c r="A21" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="15" t="str">
+      <c r="B21" s="16" t="str">
         <f aca="false">TEXT(B19,"#,##0")&amp;" ("&amp;$B$6&amp;")"&amp;IF(B20="estimate"," (estimate)","")</f>
         <v>11,000 (2021)</v>
       </c>
-      <c r="C21" s="15" t="str">
+      <c r="C21" s="16" t="str">
         <f aca="false">TEXT(C19,"#,##0")&amp;" ("&amp;$B$6&amp;")"&amp;IF(C20="estimate"," (estimate)","")</f>
         <v>10,500 (2021)</v>
       </c>
-      <c r="D21" s="15" t="str">
+      <c r="D21" s="16" t="str">
         <f aca="false">TEXT(D19,"#,##0")&amp;" ("&amp;$B$6&amp;")"&amp;IF(D20="estimate"," (estimate)","")</f>
         <v>1,400 (2021) (estimate)</v>
       </c>
-      <c r="E21" s="15" t="str">
+      <c r="E21" s="16" t="str">
         <f aca="false">TEXT(E19,"#,##0")&amp;" ("&amp;$B$6&amp;")"&amp;IF(E20="estimate"," (estimate)","")</f>
         <v>1,200 (2021)</v>
       </c>
@@ -1093,7 +1100,7 @@
       <c r="A23" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B23" s="16" t="n">
+      <c r="B23" s="17" t="n">
         <f aca="false">SUM(B19:E19)</f>
         <v>24100</v>
       </c>
@@ -1112,8 +1119,8 @@
         <v>25</v>
       </c>
       <c r="B25" s="18" t="n">
-        <f aca="false">B24*365*$B$7/1000000</f>
-        <v>43.9825</v>
+        <f aca="false">ROUND(B24,-2)</f>
+        <v>12100</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1121,27 +1128,36 @@
         <v>26</v>
       </c>
       <c r="B26" s="19" t="n">
-        <f aca="false">$B$8/B25</f>
-        <v>0.659353151821747</v>
+        <f aca="false">B25*365*$B$7/1000000</f>
+        <v>44.165</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B27" s="20" t="str">
+      <c r="B27" s="20" t="n">
+        <f aca="false">$B$8/B26</f>
+        <v>0.656628552020831</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" s="21" t="str">
         <f aca="false">IF(COUNTIF(B20:E20,"estimate")=0,"none",LEFT(IF(B20="estimate",B$10&amp;"; ","")&amp;IF(C20="estimate",C$10&amp;"; ","")&amp;IF(D20="estimate",D$10&amp;"; ","")&amp;IF(E20="estimate",E$10&amp;"; ",""),LEN(IF(B20="estimate",B$10&amp;"; ","")&amp;IF(C20="estimate",C$10&amp;"; ","")&amp;IF(D20="estimate",D$10&amp;"; ","")&amp;IF(E20="estimate",E$10&amp;"; ",""))-2))</f>
         <v>SR 1103 NW leg (Pleasant Dr)</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="21" t="s">
+      <c r="A30" s="3" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="22" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1173,12 +1189,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1189,241 +1205,241 @@
       <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" s="22" t="s">
+      <c r="B4" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="C4" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="D4" s="23" t="s">
         <v>35</v>
+      </c>
+      <c r="E4" s="23" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="C5" s="22" t="s">
+      <c r="B5" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="C5" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="E5" s="22" t="s">
+      <c r="D5" s="23" t="s">
         <v>39</v>
+      </c>
+      <c r="E5" s="23" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B6" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="B6" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="C6" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="22" t="s">
+      <c r="D6" s="23" t="s">
         <v>44</v>
+      </c>
+      <c r="E6" s="23" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B7" s="22" t="n">
+        <v>46</v>
+      </c>
+      <c r="B7" s="23" t="n">
         <v>35.25194</v>
       </c>
-      <c r="C7" s="22" t="n">
+      <c r="C7" s="23" t="n">
         <v>35.23435</v>
       </c>
-      <c r="D7" s="22" t="n">
+      <c r="D7" s="23" t="n">
         <v>35.24692</v>
       </c>
-      <c r="E7" s="22" t="n">
+      <c r="E7" s="23" t="n">
         <v>35.24582</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B8" s="22" t="n">
+        <v>47</v>
+      </c>
+      <c r="B8" s="23" t="n">
         <v>-81.50661</v>
       </c>
-      <c r="C8" s="22" t="n">
+      <c r="C8" s="23" t="n">
         <v>-81.51519</v>
       </c>
-      <c r="D8" s="22" t="n">
+      <c r="D8" s="23" t="n">
         <v>-81.50978</v>
       </c>
-      <c r="E8" s="22" t="n">
+      <c r="E8" s="23" t="n">
         <v>-81.50905</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="23" t="n">
+      <c r="A11" s="24" t="n">
         <v>2016</v>
       </c>
-      <c r="B11" s="24" t="n">
+      <c r="B11" s="25" t="n">
         <v>12000</v>
       </c>
-      <c r="C11" s="24" t="n">
+      <c r="C11" s="25" t="n">
         <v>12000</v>
       </c>
-      <c r="D11" s="24" t="n">
+      <c r="D11" s="25" t="n">
         <v>1600</v>
       </c>
-      <c r="E11" s="24"/>
+      <c r="E11" s="25"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="23" t="n">
+      <c r="A12" s="24" t="n">
         <v>2017</v>
       </c>
-      <c r="B12" s="24" t="n">
+      <c r="B12" s="25" t="n">
         <v>11000</v>
       </c>
-      <c r="C12" s="24" t="n">
+      <c r="C12" s="25" t="n">
         <v>11000</v>
       </c>
-      <c r="D12" s="24"/>
-      <c r="E12" s="24" t="n">
+      <c r="D12" s="25"/>
+      <c r="E12" s="25" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="23" t="n">
+      <c r="A13" s="24" t="n">
         <v>2018</v>
       </c>
-      <c r="B13" s="24" t="n">
+      <c r="B13" s="25" t="n">
         <v>11500</v>
       </c>
-      <c r="C13" s="24" t="n">
+      <c r="C13" s="25" t="n">
         <v>11000</v>
       </c>
-      <c r="D13" s="24" t="n">
+      <c r="D13" s="25" t="n">
         <v>1600</v>
       </c>
-      <c r="E13" s="24"/>
+      <c r="E13" s="25"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="23" t="n">
+      <c r="A14" s="24" t="n">
         <v>2019</v>
       </c>
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24" t="n">
+      <c r="B14" s="25"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="25" t="n">
         <v>1100</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="23" t="n">
+      <c r="A15" s="24" t="n">
         <v>2020</v>
       </c>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24" t="n">
+      <c r="B15" s="25"/>
+      <c r="C15" s="25" t="n">
         <v>10000</v>
       </c>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24" t="n">
+      <c r="D15" s="25"/>
+      <c r="E15" s="25" t="n">
         <v>1100</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="23" t="n">
+      <c r="A16" s="24" t="n">
         <v>2021</v>
       </c>
-      <c r="B16" s="24" t="n">
+      <c r="B16" s="25" t="n">
         <v>11000</v>
       </c>
-      <c r="C16" s="24" t="n">
+      <c r="C16" s="25" t="n">
         <v>10500</v>
       </c>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24" t="n">
+      <c r="D16" s="25"/>
+      <c r="E16" s="25" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="23" t="n">
+      <c r="A17" s="24" t="n">
         <v>2022</v>
       </c>
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24" t="n">
+      <c r="B17" s="25"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25" t="n">
         <v>1300</v>
       </c>
-      <c r="E17" s="24"/>
+      <c r="E17" s="25"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="23" t="n">
+      <c r="A18" s="24" t="n">
         <v>2023</v>
       </c>
-      <c r="B18" s="24" t="n">
+      <c r="B18" s="25" t="n">
         <v>11500</v>
       </c>
-      <c r="C18" s="24" t="n">
+      <c r="C18" s="25" t="n">
         <v>10500</v>
       </c>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24" t="n">
+      <c r="D18" s="25"/>
+      <c r="E18" s="25" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="23" t="n">
+      <c r="A19" s="24" t="n">
         <v>2024</v>
       </c>
-      <c r="B19" s="24" t="n">
+      <c r="B19" s="25" t="n">
         <v>11000</v>
       </c>
-      <c r="C19" s="24" t="n">
+      <c r="C19" s="25" t="n">
         <v>10500</v>
       </c>
-      <c r="D19" s="24" t="n">
+      <c r="D19" s="25" t="n">
         <v>1500</v>
       </c>
-      <c r="E19" s="24"/>
+      <c r="E19" s="25"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="23" t="n">
+      <c r="A20" s="24" t="n">
         <v>2025</v>
       </c>
-      <c r="B20" s="24" t="n">
+      <c r="B20" s="25" t="n">
         <v>10500</v>
       </c>
-      <c r="C20" s="24" t="n">
+      <c r="C20" s="25" t="n">
         <v>10000</v>
       </c>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24" t="n">
+      <c r="D20" s="25"/>
+      <c r="E20" s="25" t="n">
         <v>1200</v>
       </c>
     </row>
@@ -1446,7 +1462,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
@@ -1455,7 +1471,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1503,7 +1519,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B8" s="7" t="n">
         <v>22</v>
@@ -1677,40 +1693,40 @@
       <c r="A18" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="11" t="n">
-        <f aca="false">IFERROR(IF(B17&gt;=1000,ROUND(B17,-2),ROUND(B17,-1)),"")</f>
+      <c r="B18" s="14" t="n">
+        <f aca="false">IFERROR(IF(B17&gt;99999,ROUND(B17,-3),IF(B17&gt;=10000,ROUND(B17/500,0)*500,IF(B17&gt;=1000,ROUND(B17,-2),IF(B17&gt;=100,ROUND(B17/50,0)*50,ROUND(B17,-1))))),"")</f>
         <v>11000</v>
       </c>
-      <c r="C18" s="11" t="n">
-        <f aca="false">IFERROR(IF(C17&gt;=1000,ROUND(C17,-2),ROUND(C17,-1)),"")</f>
-        <v>10300</v>
-      </c>
-      <c r="D18" s="11" t="str">
-        <f aca="false">IFERROR(IF(D17&gt;=1000,ROUND(D17,-2),ROUND(D17,-1)),"")</f>
+      <c r="C18" s="14" t="n">
+        <f aca="false">IFERROR(IF(C17&gt;99999,ROUND(C17,-3),IF(C17&gt;=10000,ROUND(C17/500,0)*500,IF(C17&gt;=1000,ROUND(C17,-2),IF(C17&gt;=100,ROUND(C17/50,0)*50,ROUND(C17,-1))))),"")</f>
+        <v>10500</v>
+      </c>
+      <c r="D18" s="14" t="str">
+        <f aca="false">IFERROR(IF(D17&gt;99999,ROUND(D17,-3),IF(D17&gt;=10000,ROUND(D17/500,0)*500,IF(D17&gt;=1000,ROUND(D17,-2),IF(D17&gt;=100,ROUND(D17/50,0)*50,ROUND(D17,-1))))),"")</f>
         <v/>
       </c>
-      <c r="E18" s="11" t="n">
-        <f aca="false">IFERROR(IF(E17&gt;=1000,ROUND(E17,-2),ROUND(E17,-1)),"")</f>
+      <c r="E18" s="14" t="n">
+        <f aca="false">IFERROR(IF(E17&gt;99999,ROUND(E17,-3),IF(E17&gt;=10000,ROUND(E17/500,0)*500,IF(E17&gt;=1000,ROUND(E17,-2),IF(E17&gt;=100,ROUND(E17/50,0)*50,ROUND(E17,-1))))),"")</f>
         <v>1200</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="11" t="n">
+      <c r="B19" s="14" t="n">
         <f aca="false">IF(B12&lt;&gt;"",B12,B18)</f>
         <v>11000</v>
       </c>
-      <c r="C19" s="11" t="n">
+      <c r="C19" s="14" t="n">
         <f aca="false">IF(C12&lt;&gt;"",C12,C18)</f>
         <v>10500</v>
       </c>
-      <c r="D19" s="11" t="n">
+      <c r="D19" s="14" t="n">
         <f aca="false">IF(D12&lt;&gt;"",D12,D18)</f>
         <v>1500</v>
       </c>
-      <c r="E19" s="11" t="n">
+      <c r="E19" s="14" t="n">
         <f aca="false">IF(E12&lt;&gt;"",E12,E18)</f>
         <v>1200</v>
       </c>
@@ -1719,19 +1735,19 @@
       <c r="A20" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="15" t="str">
+      <c r="B20" s="16" t="str">
         <f aca="false">IF(B12&lt;&gt;"","count",IF(B18&lt;&gt;"","estimate","no data"))</f>
         <v>count</v>
       </c>
-      <c r="C20" s="15" t="str">
+      <c r="C20" s="16" t="str">
         <f aca="false">IF(C12&lt;&gt;"","count",IF(C18&lt;&gt;"","estimate","no data"))</f>
         <v>count</v>
       </c>
-      <c r="D20" s="15" t="str">
+      <c r="D20" s="16" t="str">
         <f aca="false">IF(D12&lt;&gt;"","count",IF(D18&lt;&gt;"","estimate","no data"))</f>
         <v>count</v>
       </c>
-      <c r="E20" s="15" t="str">
+      <c r="E20" s="16" t="str">
         <f aca="false">IF(E12&lt;&gt;"","count",IF(E18&lt;&gt;"","estimate","no data"))</f>
         <v>estimate</v>
       </c>
@@ -1740,19 +1756,19 @@
       <c r="A21" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="15" t="str">
+      <c r="B21" s="16" t="str">
         <f aca="false">TEXT(B19,"#,##0")&amp;" ("&amp;$B$6&amp;")"&amp;IF(B20="estimate"," (estimate)","")</f>
         <v>11,000 (2024)</v>
       </c>
-      <c r="C21" s="15" t="str">
+      <c r="C21" s="16" t="str">
         <f aca="false">TEXT(C19,"#,##0")&amp;" ("&amp;$B$6&amp;")"&amp;IF(C20="estimate"," (estimate)","")</f>
         <v>10,500 (2024)</v>
       </c>
-      <c r="D21" s="15" t="str">
+      <c r="D21" s="16" t="str">
         <f aca="false">TEXT(D19,"#,##0")&amp;" ("&amp;$B$6&amp;")"&amp;IF(D20="estimate"," (estimate)","")</f>
         <v>1,500 (2024)</v>
       </c>
-      <c r="E21" s="15" t="str">
+      <c r="E21" s="16" t="str">
         <f aca="false">TEXT(E19,"#,##0")&amp;" ("&amp;$B$6&amp;")"&amp;IF(E20="estimate"," (estimate)","")</f>
         <v>1,200 (2024) (estimate)</v>
       </c>
@@ -1761,7 +1777,7 @@
       <c r="A23" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B23" s="16" t="n">
+      <c r="B23" s="17" t="n">
         <f aca="false">SUM(B19:E19)</f>
         <v>24200</v>
       </c>
@@ -1780,8 +1796,8 @@
         <v>25</v>
       </c>
       <c r="B25" s="18" t="n">
-        <f aca="false">B24*365*$B$7/1000000</f>
-        <v>22.0825</v>
+        <f aca="false">ROUND(B24,-2)</f>
+        <v>12100</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1789,27 +1805,36 @@
         <v>26</v>
       </c>
       <c r="B26" s="19" t="n">
-        <f aca="false">$B$8/B25</f>
-        <v>0.99626400996264</v>
+        <f aca="false">B25*365*$B$7/1000000</f>
+        <v>22.0825</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B27" s="20" t="str">
+      <c r="B27" s="20" t="n">
+        <f aca="false">$B$8/B26</f>
+        <v>0.99626400996264</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" s="21" t="str">
         <f aca="false">IF(COUNTIF(B20:E20,"estimate")=0,"none",LEFT(IF(B20="estimate",B$10&amp;"; ","")&amp;IF(C20="estimate",C$10&amp;"; ","")&amp;IF(D20="estimate",D$10&amp;"; ","")&amp;IF(E20="estimate",E$10&amp;"; ",""),LEN(IF(B20="estimate",B$10&amp;"; ","")&amp;IF(C20="estimate",C$10&amp;"; ","")&amp;IF(D20="estimate",D$10&amp;"; ","")&amp;IF(E20="estimate",E$10&amp;"; ",""))-2))</f>
         <v>SR 1103 SE leg (Pleasant Hill Church Rd)</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="21" t="s">
-        <v>29</v>
+      <c r="A30" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="22" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>